<commit_message>
Scenariusze testowe xlsx: arkusz Informacje o 4. weryfikatorze
- "trzy weryfikatory" -> "cztery weryfikatory"
- nowy punkt listy "Odpoczynek dobowy 11h"
- link do zrodla: Weryfikatory czasu pracy/11-sto godzinny odpoczynek.md

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FG85g95PSnCDywmTxnoB4M
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Okres zatrudnienia" sheetId="2" r:id="rId2"/>
     <sheet name="Norma okresu rozliczeniowego" sheetId="3" r:id="rId3"/>
     <sheet name="Ilość dni wolnych" sheetId="4" r:id="rId4"/>
-    <sheet name="Odpoczynek dobowy 11h" sheetId="5" r:id="rId5"/>
+    <sheet name="Odpoczynek dobowy 11h" sheetId="6" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Okres zatrudnienia'!$A$4:$H$14</definedName>
@@ -32,7 +32,7 @@
     <t>Scenariusze testowe – weryfikatory czasu pracy</t>
   </si>
   <si>
-    <t>Zakres: trzy weryfikatory z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
+    <t>Zakres: cztery weryfikatory z folderu „Weryfikatory czasu pracy”, każdy na osobnym arkuszu.</t>
   </si>
   <si>
     <t/>
@@ -50,6 +50,9 @@
     <t>• Ilość dni wolnych – weryfikator kalendarza; liczba DNI WOLNYCH w okresie rozliczeniowym.</t>
   </si>
   <si>
+    <t>• Odpoczynek dobowy 11h – weryfikator dnia planu pracy; 11 h odpoczynku liczone w ramach JEDNEJ doby pracowniczej (24 h), + kontrola dnia poprzedniego.</t>
+  </si>
+  <si>
     <t>Kolumny na arkuszach scenariuszy:</t>
   </si>
   <si>
@@ -90,6 +93,9 @@
   </si>
   <si>
     <t>Weryfikatory czasu pracy/Weryfikator ilości dni okresu rozliczeniowego.md (pkt 5)</t>
+  </si>
+  <si>
+    <t>Weryfikatory czasu pracy/11-sto godzinny odpoczynek.md</t>
   </si>
   <si>
     <t>Wygenerowano: 2026-09-10</t>
@@ -1045,17 +1051,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>2</v>
+      <c r="A9" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
-        <v>7</v>
+      <c r="A10" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1086,12 +1092,12 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="s">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -1106,16 +1112,16 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="s">
-        <v>17</v>
+      <c r="A22" s="3" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1131,12 +1137,22 @@
     </row>
     <row r="26">
       <c r="A26" s="3" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="s">
-        <v>21</v>
+      <c r="A27" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1159,58 +1175,58 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" ht="30">
       <c r="A5" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>2</v>
@@ -1221,22 +1237,22 @@
     </row>
     <row r="6" ht="30">
       <c r="A6" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="F6" s="8" t="s">
         <v>39</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>37</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>2</v>
@@ -1247,22 +1263,22 @@
     </row>
     <row r="7" ht="30">
       <c r="A7" s="7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>41</v>
-      </c>
       <c r="E7" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>2</v>
@@ -1273,22 +1289,22 @@
     </row>
     <row r="8" ht="30">
       <c r="A8" s="7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>2</v>
@@ -1299,22 +1315,22 @@
     </row>
     <row r="9" ht="30">
       <c r="A9" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="E9" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>49</v>
-      </c>
       <c r="F9" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>2</v>
@@ -1325,22 +1341,22 @@
     </row>
     <row r="10" ht="45">
       <c r="A10" s="7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>2</v>
@@ -1351,22 +1367,22 @@
     </row>
     <row r="11" ht="30">
       <c r="A11" s="7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>2</v>
@@ -1377,22 +1393,22 @@
     </row>
     <row r="12" ht="30">
       <c r="A12" s="7" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>2</v>
@@ -1403,22 +1419,22 @@
     </row>
     <row r="13" ht="30">
       <c r="A13" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>2</v>
@@ -1429,22 +1445,22 @@
     </row>
     <row r="14" ht="45">
       <c r="A14" s="7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G14" s="11" t="s">
         <v>2</v>
@@ -1474,58 +1490,58 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>2</v>
@@ -1536,22 +1552,22 @@
     </row>
     <row r="6" ht="75">
       <c r="A6" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>2</v>
@@ -1562,22 +1578,22 @@
     </row>
     <row r="7" ht="60">
       <c r="A7" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>84</v>
-      </c>
       <c r="F7" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>2</v>
@@ -1588,22 +1604,22 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>2</v>
@@ -1614,22 +1630,22 @@
     </row>
     <row r="9" ht="45">
       <c r="A9" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>2</v>
@@ -1640,22 +1656,22 @@
     </row>
     <row r="10" ht="75">
       <c r="A10" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>2</v>
@@ -1686,64 +1702,64 @@
   <sheetData>
     <row r="1" ht="17.25">
       <c r="A1" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>2</v>
@@ -1754,25 +1770,25 @@
     </row>
     <row r="6" ht="45">
       <c r="A6" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>110</v>
-      </c>
       <c r="G6" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>2</v>
@@ -1783,25 +1799,25 @@
     </row>
     <row r="7" ht="36">
       <c r="A7" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>2</v>
@@ -1812,25 +1828,25 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="7" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>2</v>
@@ -1841,25 +1857,25 @@
     </row>
     <row r="9" ht="75">
       <c r="A9" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>2</v>
@@ -1870,25 +1886,25 @@
     </row>
     <row r="10" ht="60">
       <c r="A10" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>2</v>
@@ -1899,25 +1915,25 @@
     </row>
     <row r="11" ht="48">
       <c r="A11" s="7" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>2</v>
@@ -1948,7 +1964,7 @@
   <sheetData>
     <row r="1" ht="15.75">
       <c r="A1" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
@@ -1961,7 +1977,7 @@
     </row>
     <row r="2" ht="16.8" customHeight="1">
       <c r="A2" s="14" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="14"/>
@@ -1974,54 +1990,54 @@
     </row>
     <row r="4" ht="7.2" customHeight="1">
       <c r="A4" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" ht="45">
       <c r="A5" s="16" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H5" s="16" t="s">
         <v>2</v>
@@ -2032,25 +2048,25 @@
     </row>
     <row r="6" ht="45">
       <c r="A6" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>36</v>
-      </c>
       <c r="G6" s="16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H6" s="16" t="s">
         <v>2</v>
@@ -2061,25 +2077,25 @@
     </row>
     <row r="7" ht="45">
       <c r="A7" s="16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C7" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="D7" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="D7" s="16" t="s">
-        <v>148</v>
-      </c>
       <c r="E7" s="16" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H7" s="16" t="s">
         <v>2</v>
@@ -2090,25 +2106,25 @@
     </row>
     <row r="8" ht="45">
       <c r="A8" s="16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B8" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="E8" s="16" t="s">
-        <v>151</v>
-      </c>
       <c r="F8" s="16" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H8" s="16" t="s">
         <v>2</v>
@@ -2119,25 +2135,25 @@
     </row>
     <row r="9" ht="45">
       <c r="A9" s="16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H9" s="16" t="s">
         <v>2</v>
@@ -2148,25 +2164,25 @@
     </row>
     <row r="10" ht="45">
       <c r="A10" s="16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>2</v>
@@ -2177,25 +2193,25 @@
     </row>
     <row r="11" ht="30">
       <c r="A11" s="16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H11" s="16" t="s">
         <v>2</v>
@@ -2206,25 +2222,25 @@
     </row>
     <row r="12" ht="30">
       <c r="A12" s="16" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H12" s="16" t="s">
         <v>2</v>
@@ -2235,25 +2251,25 @@
     </row>
     <row r="13" ht="30">
       <c r="A13" s="16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H13" s="16" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Weryfikator 11h odpoczynek: dociąganie wczesnorannych stref dnia następnego
Zgłoszenie: sobota 8:00-21:00 + niedziela 7:00-20:00 nie dawało komunikatu,
mimo że realny odpoczynek to tylko 10h. Przyczyna: każda doba liczyła
przerwę wyłącznie ze stref własnego dnia, więc doba soboty i doba niedzieli
liczone osobno dawały po 11:00 (dokładnie na granicy) - luka opisana
wcześniej w .md jako "do decyzji, czy rozszerzać".

Fix: dociągamy wczesnoranne strefy dnia następnego (przesunięte o +24h),
które wpadają w okno bieżącej doby - przycinane tą samą logiką klipowania
co reszta stref. Dodano scenariusz 10 do arkusza testowego.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ck4fdapYvFNYgqnSzew24s
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -569,6 +569,24 @@
   </si>
   <si>
     <t>Brak błędu z tytułu doby D-1</t>
+  </si>
+  <si>
+    <t>Sobota: Praca w normie 8:00-21:00; Niedziela: Praca w normie 7:00-20:00 (wczesnoranna strefa dnia następnego wpada w okno doby sobotniej)</t>
+  </si>
+  <si>
+    <t>D0 soboty = 8:00, okno doby = [8:00 sob. ; 8:00 niedz.]. Fragment niedzieli 7:00-8:00 dociągnięty do tej doby (przesunięty o +24h). Ostatnia strefa soboty kończy się 21:00 -&gt; przerwa końcowa liczona do początku dociągniętej strefy niedzieli (7:00 niedz. = 31:00 na osi doby) = 21:00-&gt;7:00 = 10:00.</t>
+  </si>
+  <si>
+    <t>sobota (oraz niedziela - kontrola dnia poprzedniego)</t>
+  </si>
+  <si>
+    <t>BŁĄD (10:00 &lt; 11:00) - licząc każdą dobę tylko z własnych stref (bez dociągania dnia następnego) wychodziłoby błędnie 11:00 w obu dobach, czyli brak błędu</t>
+  </si>
+  <si>
+    <t>nie zachowano wymaganego przepisami prawa pracy 11-godzinnego odpoczynku dobowego (najdłuższa przerwa w dobie: 10:00)</t>
+  </si>
+  <si>
+    <t>Zgłoszone przez użytkownika jako brak komunikatu; usunięto znane ograniczenie - dodano dociąganie wczesnorannych stref dnia następnego do okna doby (patrz .md, commit fix)</t>
   </si>
 </sst>
 </file>
@@ -2278,6 +2296,35 @@
         <v>2</v>
       </c>
     </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C14" t="s">
+        <v>178</v>
+      </c>
+      <c r="D14" t="s">
+        <v>179</v>
+      </c>
+      <c r="E14" t="s">
+        <v>180</v>
+      </c>
+      <c r="F14" t="s">
+        <v>181</v>
+      </c>
+      <c r="G14" t="s">
+        <v>39</v>
+      </c>
+      <c r="H14" t="s">
+        <v>2</v>
+      </c>
+      <c r="I14" t="s">
+        <v>182</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:I13"/>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Weryfikator 11h odpoczynek: zamknięcie zadania po teście w GUI
Test w GUI klienta 2026-09-11 potwierdził poprawność fixu (dociąganie
wczesnorannych stref dnia następnego, commit 0588e59). Zweryfikowano
scenariusz sobota 8:00-21:00 / niedziela 7:00-20:00.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ck4fdapYvFNYgqnSzew24s
</commit_message>
<xml_diff>
--- a/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
+++ b/Weryfikatory czasu pracy/Scenariusze testowe weryfikatorow czasu pracy.xlsx
@@ -586,7 +586,13 @@
     <t>nie zachowano wymaganego przepisami prawa pracy 11-godzinnego odpoczynku dobowego (najdłuższa przerwa w dobie: 10:00)</t>
   </si>
   <si>
-    <t>Zgłoszone przez użytkownika jako brak komunikatu; usunięto znane ograniczenie - dodano dociąganie wczesnorannych stref dnia następnego do okna doby (patrz .md, commit fix)</t>
+    <t>Tak (2026-09-11)</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Zgłoszone przez użytkownika jako brak komunikatu; usunięto znane ograniczenie - dodano dociąganie wczesnorannych stref dnia następnego do okna doby (patrz .md, commit fix) Zweryfikowano w GUI klienta 2026-09-11 - komunikat pojawia się poprawnie. Zadanie zamknięte.</t>
   </si>
 </sst>
 </file>
@@ -2316,13 +2322,13 @@
         <v>181</v>
       </c>
       <c r="G14" t="s">
-        <v>39</v>
+        <v>182</v>
       </c>
       <c r="H14" t="s">
-        <v>2</v>
+        <v>183</v>
       </c>
       <c r="I14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>